<commit_message>
feat: Enhance menu and vendor management functionality
- Added method to add items to cart by name in MenuPage.
- Implemented QR code page with navigation and display checks in PickupQrPage.
- Expanded VendorMenuManagePage with item creation, validation, and duplicate handling.
- Introduced WalletPage enhancements for transaction timestamps and logout checks.
- Improved ExtentReportManager for report directory management.
- Updated ScreenshotUtils to utilize report directory for screenshots.
- Refactored DefectRegressionTests for better structure and added new test cases.
- Created VendorQueuePage to manage vendor queue states and visibility.
- Updated testng.xml for streamlined test execution and parallelization.
</commit_message>
<xml_diff>
--- a/Deliverables/Functional Testing Report for Cafetron.xlsx
+++ b/Deliverables/Functional Testing Report for Cafetron.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2492171_cognizant_com/Documents/Documents/Cafetronnnnnnnn/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2492171_cognizant_com/Documents/Documents/CAFETRON_TESTING/Deliverables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="126" documentId="13_ncr:1_{93FE7E23-1C99-4CD5-869C-5B188F6F59A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9A8CAD5-F5DB-4118-9D65-DC2D5721CDAC}"/>
+  <xr:revisionPtr revIDLastSave="127" documentId="13_ncr:1_{93FE7E23-1C99-4CD5-869C-5B188F6F59A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69EBACE1-22B0-4419-BE35-81CB30FB23B9}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2188" uniqueCount="1018">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2188" uniqueCount="1013">
   <si>
     <t>Note</t>
   </si>
@@ -1564,12 +1564,6 @@
   </si>
   <si>
     <t>DF-022</t>
-  </si>
-  <si>
-    <t>Verify over-stock checkout error appears in Cards flow</t>
-  </si>
-  <si>
-    <t>Employee cart quantity exceeds stock.</t>
   </si>
   <si>
     <t>Verify pickup QR page has back navigation</t>
@@ -2913,21 +2907,6 @@
   </si>
   <si>
     <t>1. Cart allowed quantity 9 and showed total Rs 225.00 without stock warning.</t>
-  </si>
-  <si>
-    <t>1. Open checkout.
-2. Select Dinner slot.
-3. Continue through Cards checkout to Place order.
-4. Click Place Order.
-5. Observe error location.
-6. Switch to Overview.</t>
-  </si>
-  <si>
-    <t>1. Stock error should be shown immediately near Place Order in Cards flow.
-2. User should not need to switch tabs to see the error.</t>
-  </si>
-  <si>
-    <t>1. Cards flow showed Placing Order without visible error; Insufficient stock appeared only after switching to Overview.</t>
   </si>
   <si>
     <t>1. Login as employee.
@@ -4859,10 +4838,10 @@
         <v>182</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>949</v>
+        <v>944</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>950</v>
+        <v>945</v>
       </c>
       <c r="E30" s="7" t="s">
         <v>46</v>
@@ -5242,13 +5221,13 @@
         <v>242</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>647</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>649</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>650</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>651</v>
       </c>
       <c r="H2" s="9" t="s">
         <v>243</v>
@@ -5274,13 +5253,13 @@
         <v>247</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>650</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>651</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>652</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>653</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>654</v>
       </c>
       <c r="H3" s="9" t="s">
         <v>243</v>
@@ -5306,13 +5285,13 @@
         <v>249</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>653</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="G4" s="9" t="s">
         <v>655</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>656</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>657</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>243</v>
@@ -5338,13 +5317,13 @@
         <v>251</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>656</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>657</v>
+      </c>
+      <c r="G5" s="9" t="s">
         <v>658</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>659</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>660</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>243</v>
@@ -5364,19 +5343,19 @@
         <v>62</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>251</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>661</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>662</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>663</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>664</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>243</v>
@@ -5385,7 +5364,7 @@
         <v>244</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
@@ -5402,13 +5381,13 @@
         <v>255</v>
       </c>
       <c r="E7" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>665</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>666</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>667</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>668</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>243</v>
@@ -5434,13 +5413,13 @@
         <v>257</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>667</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>669</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>671</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>243</v>
@@ -5466,13 +5445,13 @@
         <v>259</v>
       </c>
       <c r="E9" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>671</v>
+      </c>
+      <c r="G9" s="9" t="s">
         <v>672</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>673</v>
-      </c>
-      <c r="G9" s="9" t="s">
-        <v>674</v>
       </c>
       <c r="H9" s="9" t="s">
         <v>243</v>
@@ -5498,13 +5477,13 @@
         <v>261</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>262</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>243</v>
@@ -5530,13 +5509,13 @@
         <v>261</v>
       </c>
       <c r="E11" s="3" t="s">
+        <v>675</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>676</v>
+      </c>
+      <c r="G11" s="9" t="s">
         <v>677</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>678</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>679</v>
       </c>
       <c r="H11" s="9" t="s">
         <v>243</v>
@@ -5562,13 +5541,13 @@
         <v>265</v>
       </c>
       <c r="E12" s="3" t="s">
+        <v>678</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>679</v>
+      </c>
+      <c r="G12" s="9" t="s">
         <v>680</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>681</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>682</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>243</v>
@@ -5594,13 +5573,13 @@
         <v>267</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="H13" s="9" t="s">
         <v>243</v>
@@ -5626,13 +5605,13 @@
         <v>269</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>885</v>
+        <v>880</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>243</v>
@@ -5658,13 +5637,13 @@
         <v>271</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>887</v>
+        <v>882</v>
       </c>
       <c r="H15" s="9" t="s">
         <v>243</v>
@@ -5690,13 +5669,13 @@
         <v>269</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>888</v>
+        <v>883</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>243</v>
@@ -5705,7 +5684,7 @@
         <v>244</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -5722,13 +5701,13 @@
         <v>274</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>891</v>
+        <v>886</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>892</v>
+        <v>887</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>243</v>
@@ -5754,13 +5733,13 @@
         <v>284</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>243</v>
@@ -5786,13 +5765,13 @@
         <v>284</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>277</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>894</v>
+        <v>889</v>
       </c>
       <c r="H19" s="9" t="s">
         <v>243</v>
@@ -5818,13 +5797,13 @@
         <v>279</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>895</v>
+        <v>890</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>243</v>
@@ -5850,13 +5829,13 @@
         <v>281</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="H21" s="9" t="s">
         <v>243</v>
@@ -5876,19 +5855,19 @@
         <v>78</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>282</v>
       </c>
       <c r="E22" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>697</v>
+      </c>
+      <c r="G22" s="9" t="s">
         <v>698</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>699</v>
-      </c>
-      <c r="G22" s="9" t="s">
-        <v>700</v>
       </c>
       <c r="H22" s="9" t="s">
         <v>243</v>
@@ -5897,7 +5876,7 @@
         <v>244</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>897</v>
+        <v>892</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -5914,13 +5893,13 @@
         <v>284</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>898</v>
+        <v>893</v>
       </c>
       <c r="H23" s="9" t="s">
         <v>243</v>
@@ -5929,7 +5908,7 @@
         <v>244</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>899</v>
+        <v>894</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="58" x14ac:dyDescent="0.35">
@@ -5946,13 +5925,13 @@
         <v>284</v>
       </c>
       <c r="E24" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>702</v>
+      </c>
+      <c r="G24" s="9" t="s">
         <v>703</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>704</v>
-      </c>
-      <c r="G24" s="9" t="s">
-        <v>705</v>
       </c>
       <c r="H24" s="9" t="s">
         <v>243</v>
@@ -5978,13 +5957,13 @@
         <v>284</v>
       </c>
       <c r="E25" s="3" t="s">
+        <v>704</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>705</v>
+      </c>
+      <c r="G25" s="9" t="s">
         <v>706</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>707</v>
-      </c>
-      <c r="G25" s="9" t="s">
-        <v>708</v>
       </c>
       <c r="H25" s="9" t="s">
         <v>243</v>
@@ -6010,13 +5989,13 @@
         <v>284</v>
       </c>
       <c r="E26" s="3" t="s">
+        <v>707</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="G26" s="9" t="s">
         <v>709</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>710</v>
-      </c>
-      <c r="G26" s="9" t="s">
-        <v>711</v>
       </c>
       <c r="H26" s="9" t="s">
         <v>243</v>
@@ -6042,13 +6021,13 @@
         <v>290</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>291</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>900</v>
+        <v>895</v>
       </c>
       <c r="H27" s="9" t="s">
         <v>243</v>
@@ -6074,13 +6053,13 @@
         <v>293</v>
       </c>
       <c r="E28" s="3" t="s">
+        <v>711</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>712</v>
+      </c>
+      <c r="G28" s="9" t="s">
         <v>713</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>714</v>
-      </c>
-      <c r="G28" s="9" t="s">
-        <v>715</v>
       </c>
       <c r="H28" s="9" t="s">
         <v>243</v>
@@ -6106,13 +6085,13 @@
         <v>295</v>
       </c>
       <c r="E29" s="3" t="s">
+        <v>714</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>715</v>
+      </c>
+      <c r="G29" s="9" t="s">
         <v>716</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>717</v>
-      </c>
-      <c r="G29" s="9" t="s">
-        <v>718</v>
       </c>
       <c r="H29" s="9" t="s">
         <v>243</v>
@@ -6138,13 +6117,13 @@
         <v>297</v>
       </c>
       <c r="E30" s="3" t="s">
+        <v>717</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>718</v>
+      </c>
+      <c r="G30" s="9" t="s">
         <v>719</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>720</v>
-      </c>
-      <c r="G30" s="9" t="s">
-        <v>721</v>
       </c>
       <c r="H30" s="9" t="s">
         <v>243</v>
@@ -6170,13 +6149,13 @@
         <v>299</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>300</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>901</v>
+        <v>896</v>
       </c>
       <c r="H31" s="9" t="s">
         <v>252</v>
@@ -6202,13 +6181,13 @@
         <v>267</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>902</v>
+        <v>897</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="H32" s="9" t="s">
         <v>243</v>
@@ -6234,13 +6213,13 @@
         <v>304</v>
       </c>
       <c r="E33" s="3" t="s">
+        <v>723</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>724</v>
+      </c>
+      <c r="G33" s="9" t="s">
         <v>725</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>726</v>
-      </c>
-      <c r="G33" s="9" t="s">
-        <v>727</v>
       </c>
       <c r="H33" s="9" t="s">
         <v>243</v>
@@ -6266,13 +6245,13 @@
         <v>306</v>
       </c>
       <c r="E34" s="3" t="s">
+        <v>726</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>727</v>
+      </c>
+      <c r="G34" s="9" t="s">
         <v>728</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>729</v>
-      </c>
-      <c r="G34" s="9" t="s">
-        <v>730</v>
       </c>
       <c r="H34" s="9" t="s">
         <v>243</v>
@@ -6298,13 +6277,13 @@
         <v>309</v>
       </c>
       <c r="E35" s="3" t="s">
+        <v>729</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>730</v>
+      </c>
+      <c r="G35" s="9" t="s">
         <v>731</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>732</v>
-      </c>
-      <c r="G35" s="9" t="s">
-        <v>733</v>
       </c>
       <c r="H35" s="9" t="s">
         <v>243</v>
@@ -6330,13 +6309,13 @@
         <v>309</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="H36" s="9" t="s">
         <v>243</v>
@@ -6362,13 +6341,13 @@
         <v>309</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="H37" s="9" t="s">
         <v>243</v>
@@ -6394,13 +6373,13 @@
         <v>317</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>904</v>
+        <v>899</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>903</v>
+        <v>898</v>
       </c>
       <c r="H38" s="9" t="s">
         <v>243</v>
@@ -6426,13 +6405,13 @@
         <v>320</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>906</v>
+        <v>901</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="H39" s="9" t="s">
         <v>243</v>
@@ -6458,13 +6437,13 @@
         <v>320</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>323</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="H40" s="9" t="s">
         <v>243</v>
@@ -6490,13 +6469,13 @@
         <v>326</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>907</v>
+        <v>902</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="H41" s="9" t="s">
         <v>243</v>
@@ -6522,13 +6501,13 @@
         <v>329</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>330</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="H42" s="9" t="s">
         <v>243</v>
@@ -6548,28 +6527,28 @@
         <v>321</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>926</v>
+        <v>921</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>333</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>927</v>
+        <v>922</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>928</v>
+        <v>923</v>
       </c>
       <c r="G43" s="9" t="s">
-        <v>929</v>
+        <v>924</v>
       </c>
       <c r="H43" s="9" t="s">
         <v>252</v>
       </c>
       <c r="I43" s="9" t="s">
-        <v>920</v>
+        <v>915</v>
       </c>
       <c r="J43" s="9" t="s">
-        <v>930</v>
+        <v>925</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="58" x14ac:dyDescent="0.35">
@@ -6586,13 +6565,13 @@
         <v>333</v>
       </c>
       <c r="E44" s="3" t="s">
+        <v>745</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>746</v>
+      </c>
+      <c r="G44" s="9" t="s">
         <v>747</v>
-      </c>
-      <c r="F44" s="3" t="s">
-        <v>748</v>
-      </c>
-      <c r="G44" s="9" t="s">
-        <v>749</v>
       </c>
       <c r="H44" s="9" t="s">
         <v>243</v>
@@ -6618,13 +6597,13 @@
         <v>340</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>341</v>
       </c>
       <c r="G45" s="9" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="H45" s="9" t="s">
         <v>252</v>
@@ -6633,7 +6612,7 @@
         <v>342</v>
       </c>
       <c r="J45" s="9" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="58" x14ac:dyDescent="0.35">
@@ -6650,13 +6629,13 @@
         <v>345</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>346</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="H46" s="9" t="s">
         <v>243</v>
@@ -6682,13 +6661,13 @@
         <v>333</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>349</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="H47" s="9" t="s">
         <v>243</v>
@@ -6714,13 +6693,13 @@
         <v>352</v>
       </c>
       <c r="E48" s="3" t="s">
+        <v>754</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>755</v>
+      </c>
+      <c r="G48" s="9" t="s">
         <v>756</v>
-      </c>
-      <c r="F48" s="3" t="s">
-        <v>757</v>
-      </c>
-      <c r="G48" s="9" t="s">
-        <v>758</v>
       </c>
       <c r="H48" s="9" t="s">
         <v>243</v>
@@ -6746,13 +6725,13 @@
         <v>355</v>
       </c>
       <c r="E49" s="3" t="s">
+        <v>757</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>758</v>
+      </c>
+      <c r="G49" s="9" t="s">
         <v>759</v>
-      </c>
-      <c r="F49" s="3" t="s">
-        <v>760</v>
-      </c>
-      <c r="G49" s="9" t="s">
-        <v>761</v>
       </c>
       <c r="H49" s="9" t="s">
         <v>243</v>
@@ -6778,13 +6757,13 @@
         <v>352</v>
       </c>
       <c r="E50" s="3" t="s">
+        <v>760</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="G50" s="9" t="s">
         <v>762</v>
-      </c>
-      <c r="F50" s="3" t="s">
-        <v>763</v>
-      </c>
-      <c r="G50" s="9" t="s">
-        <v>764</v>
       </c>
       <c r="H50" s="9" t="s">
         <v>243</v>
@@ -6810,13 +6789,13 @@
         <v>360</v>
       </c>
       <c r="E51" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>764</v>
+      </c>
+      <c r="G51" s="9" t="s">
         <v>765</v>
-      </c>
-      <c r="F51" s="3" t="s">
-        <v>766</v>
-      </c>
-      <c r="G51" s="9" t="s">
-        <v>767</v>
       </c>
       <c r="H51" s="9" t="s">
         <v>243</v>
@@ -6842,13 +6821,13 @@
         <v>360</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>909</v>
+        <v>904</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>910</v>
+        <v>905</v>
       </c>
       <c r="H52" s="9" t="s">
         <v>243</v>
@@ -6874,13 +6853,13 @@
         <v>365</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="F53" s="3" t="s">
         <v>366</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="H53" s="9" t="s">
         <v>243</v>
@@ -6906,22 +6885,22 @@
         <v>369</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>912</v>
+        <v>907</v>
       </c>
       <c r="H54" s="9" t="s">
         <v>252</v>
       </c>
       <c r="I54" s="9" t="s">
-        <v>913</v>
+        <v>908</v>
       </c>
       <c r="J54" s="9" t="s">
-        <v>914</v>
+        <v>909</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -6938,13 +6917,13 @@
         <v>333</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>918</v>
+        <v>913</v>
       </c>
       <c r="H55" s="9" t="s">
         <v>243</v>
@@ -6970,13 +6949,13 @@
         <v>374</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>375</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="H56" s="9" t="s">
         <v>243</v>
@@ -7002,13 +6981,13 @@
         <v>378</v>
       </c>
       <c r="E57" s="3" t="s">
+        <v>774</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>775</v>
+      </c>
+      <c r="G57" s="9" t="s">
         <v>776</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>777</v>
-      </c>
-      <c r="G57" s="9" t="s">
-        <v>778</v>
       </c>
       <c r="H57" s="9" t="s">
         <v>243</v>
@@ -7034,13 +7013,13 @@
         <v>381</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>382</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="H58" s="9" t="s">
         <v>243</v>
@@ -7066,13 +7045,13 @@
         <v>384</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="F59" s="3" t="s">
         <v>387</v>
       </c>
       <c r="G59" s="9" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="H59" s="9" t="s">
         <v>243</v>
@@ -7104,16 +7083,16 @@
         <v>391</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>931</v>
+        <v>926</v>
       </c>
       <c r="H60" s="9" t="s">
         <v>252</v>
       </c>
       <c r="I60" s="9" t="s">
-        <v>919</v>
+        <v>914</v>
       </c>
       <c r="J60" s="9" t="s">
-        <v>932</v>
+        <v>927</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -7130,13 +7109,13 @@
         <v>394</v>
       </c>
       <c r="E61" s="3" t="s">
+        <v>781</v>
+      </c>
+      <c r="F61" s="3" t="s">
+        <v>782</v>
+      </c>
+      <c r="G61" s="9" t="s">
         <v>783</v>
-      </c>
-      <c r="F61" s="3" t="s">
-        <v>784</v>
-      </c>
-      <c r="G61" s="9" t="s">
-        <v>785</v>
       </c>
       <c r="H61" s="9" t="s">
         <v>243</v>
@@ -7162,13 +7141,13 @@
         <v>397</v>
       </c>
       <c r="E62" s="3" t="s">
+        <v>784</v>
+      </c>
+      <c r="F62" s="3" t="s">
+        <v>785</v>
+      </c>
+      <c r="G62" s="9" t="s">
         <v>786</v>
-      </c>
-      <c r="F62" s="3" t="s">
-        <v>787</v>
-      </c>
-      <c r="G62" s="9" t="s">
-        <v>788</v>
       </c>
       <c r="H62" s="9" t="s">
         <v>243</v>
@@ -7177,7 +7156,7 @@
         <v>244</v>
       </c>
       <c r="J62" s="9" t="s">
-        <v>921</v>
+        <v>916</v>
       </c>
     </row>
     <row r="63" spans="1:10" ht="58" x14ac:dyDescent="0.35">
@@ -7194,22 +7173,22 @@
         <v>400</v>
       </c>
       <c r="E63" s="3" t="s">
+        <v>787</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>788</v>
+      </c>
+      <c r="G63" s="9" t="s">
         <v>789</v>
-      </c>
-      <c r="F63" s="3" t="s">
-        <v>790</v>
-      </c>
-      <c r="G63" s="9" t="s">
-        <v>791</v>
       </c>
       <c r="H63" s="9" t="s">
         <v>252</v>
       </c>
       <c r="I63" s="9" t="s">
-        <v>933</v>
+        <v>928</v>
       </c>
       <c r="J63" s="9" t="s">
-        <v>934</v>
+        <v>929</v>
       </c>
     </row>
     <row r="64" spans="1:10" ht="87" x14ac:dyDescent="0.35">
@@ -7226,22 +7205,22 @@
         <v>394</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>403</v>
       </c>
       <c r="G64" s="9" t="s">
-        <v>935</v>
+        <v>930</v>
       </c>
       <c r="H64" s="9" t="s">
         <v>252</v>
       </c>
       <c r="I64" s="9" t="s">
-        <v>936</v>
+        <v>931</v>
       </c>
       <c r="J64" s="9" t="s">
-        <v>934</v>
+        <v>929</v>
       </c>
     </row>
     <row r="65" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -7258,13 +7237,13 @@
         <v>381</v>
       </c>
       <c r="E65" s="3" t="s">
+        <v>791</v>
+      </c>
+      <c r="F65" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="G65" s="9" t="s">
         <v>793</v>
-      </c>
-      <c r="F65" s="3" t="s">
-        <v>794</v>
-      </c>
-      <c r="G65" s="9" t="s">
-        <v>795</v>
       </c>
       <c r="H65" s="9" t="s">
         <v>243</v>
@@ -7290,22 +7269,22 @@
         <v>408</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="G66" s="9" t="s">
-        <v>937</v>
+        <v>932</v>
       </c>
       <c r="H66" s="9" t="s">
         <v>252</v>
       </c>
       <c r="I66" s="9" t="s">
-        <v>922</v>
+        <v>917</v>
       </c>
       <c r="J66" s="9" t="s">
-        <v>938</v>
+        <v>933</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="58" x14ac:dyDescent="0.35">
@@ -7322,13 +7301,13 @@
         <v>411</v>
       </c>
       <c r="E67" s="3" t="s">
+        <v>796</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>797</v>
+      </c>
+      <c r="G67" s="9" t="s">
         <v>798</v>
-      </c>
-      <c r="F67" s="3" t="s">
-        <v>799</v>
-      </c>
-      <c r="G67" s="9" t="s">
-        <v>800</v>
       </c>
       <c r="H67" s="9" t="s">
         <v>243</v>
@@ -7354,13 +7333,13 @@
         <v>417</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="F68" s="3" t="s">
         <v>418</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="H68" s="9" t="s">
         <v>243</v>
@@ -7386,13 +7365,13 @@
         <v>417</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="F69" s="3" t="s">
         <v>421</v>
       </c>
       <c r="G69" s="9" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="H69" s="9" t="s">
         <v>243</v>
@@ -7412,28 +7391,28 @@
         <v>398</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>939</v>
+        <v>934</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>940</v>
+        <v>935</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>941</v>
+        <v>936</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>942</v>
+        <v>937</v>
       </c>
       <c r="G70" s="9" t="s">
-        <v>943</v>
+        <v>938</v>
       </c>
       <c r="H70" s="9" t="s">
         <v>252</v>
       </c>
       <c r="I70" s="9" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
       <c r="J70" s="9" t="s">
-        <v>944</v>
+        <v>939</v>
       </c>
     </row>
     <row r="71" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
@@ -7450,13 +7429,13 @@
         <v>333</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="F71" s="3" t="s">
         <v>425</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="H71" s="9" t="s">
         <v>243</v>
@@ -7482,13 +7461,13 @@
         <v>381</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="F72" s="3" t="s">
         <v>428</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="H72" s="9" t="s">
         <v>243</v>
@@ -7514,13 +7493,13 @@
         <v>267</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="F73" s="3" t="s">
         <v>431</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="H73" s="9" t="s">
         <v>243</v>
@@ -7546,13 +7525,13 @@
         <v>434</v>
       </c>
       <c r="E74" s="3" t="s">
+        <v>809</v>
+      </c>
+      <c r="F74" s="3" t="s">
+        <v>810</v>
+      </c>
+      <c r="G74" s="9" t="s">
         <v>811</v>
-      </c>
-      <c r="F74" s="3" t="s">
-        <v>812</v>
-      </c>
-      <c r="G74" s="9" t="s">
-        <v>813</v>
       </c>
       <c r="H74" s="9" t="s">
         <v>243</v>
@@ -7578,13 +7557,13 @@
         <v>438</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
       <c r="F75" s="3" t="s">
         <v>439</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="H75" s="9" t="s">
         <v>243</v>
@@ -7610,13 +7589,13 @@
         <v>442</v>
       </c>
       <c r="E76" s="3" t="s">
+        <v>814</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>815</v>
+      </c>
+      <c r="G76" s="9" t="s">
         <v>816</v>
-      </c>
-      <c r="F76" s="3" t="s">
-        <v>817</v>
-      </c>
-      <c r="G76" s="9" t="s">
-        <v>818</v>
       </c>
       <c r="H76" s="9" t="s">
         <v>243</v>
@@ -7642,13 +7621,13 @@
         <v>442</v>
       </c>
       <c r="E77" s="3" t="s">
+        <v>817</v>
+      </c>
+      <c r="F77" s="3" t="s">
+        <v>818</v>
+      </c>
+      <c r="G77" s="9" t="s">
         <v>819</v>
-      </c>
-      <c r="F77" s="3" t="s">
-        <v>820</v>
-      </c>
-      <c r="G77" s="9" t="s">
-        <v>821</v>
       </c>
       <c r="H77" s="9" t="s">
         <v>243</v>
@@ -7674,13 +7653,13 @@
         <v>446</v>
       </c>
       <c r="E78" s="3" t="s">
+        <v>820</v>
+      </c>
+      <c r="F78" s="3" t="s">
+        <v>821</v>
+      </c>
+      <c r="G78" s="9" t="s">
         <v>822</v>
-      </c>
-      <c r="F78" s="3" t="s">
-        <v>823</v>
-      </c>
-      <c r="G78" s="9" t="s">
-        <v>824</v>
       </c>
       <c r="H78" s="9" t="s">
         <v>252</v>
@@ -7706,13 +7685,13 @@
         <v>452</v>
       </c>
       <c r="E79" s="3" t="s">
+        <v>823</v>
+      </c>
+      <c r="F79" s="3" t="s">
+        <v>824</v>
+      </c>
+      <c r="G79" s="9" t="s">
         <v>825</v>
-      </c>
-      <c r="F79" s="3" t="s">
-        <v>826</v>
-      </c>
-      <c r="G79" s="9" t="s">
-        <v>827</v>
       </c>
       <c r="H79" s="9" t="s">
         <v>252</v>
@@ -7738,13 +7717,13 @@
         <v>452</v>
       </c>
       <c r="E80" s="3" t="s">
+        <v>826</v>
+      </c>
+      <c r="F80" s="3" t="s">
+        <v>827</v>
+      </c>
+      <c r="G80" s="9" t="s">
         <v>828</v>
-      </c>
-      <c r="F80" s="3" t="s">
-        <v>829</v>
-      </c>
-      <c r="G80" s="9" t="s">
-        <v>830</v>
       </c>
       <c r="H80" s="9" t="s">
         <v>252</v>
@@ -7770,13 +7749,13 @@
         <v>446</v>
       </c>
       <c r="E81" s="3" t="s">
+        <v>829</v>
+      </c>
+      <c r="F81" s="3" t="s">
+        <v>830</v>
+      </c>
+      <c r="G81" s="9" t="s">
         <v>831</v>
-      </c>
-      <c r="F81" s="3" t="s">
-        <v>832</v>
-      </c>
-      <c r="G81" s="9" t="s">
-        <v>833</v>
       </c>
       <c r="H81" s="9" t="s">
         <v>252</v>
@@ -7802,13 +7781,13 @@
         <v>452</v>
       </c>
       <c r="E82" s="3" t="s">
+        <v>832</v>
+      </c>
+      <c r="F82" s="3" t="s">
+        <v>833</v>
+      </c>
+      <c r="G82" s="9" t="s">
         <v>834</v>
-      </c>
-      <c r="F82" s="3" t="s">
-        <v>835</v>
-      </c>
-      <c r="G82" s="9" t="s">
-        <v>836</v>
       </c>
       <c r="H82" s="9" t="s">
         <v>252</v>
@@ -7834,13 +7813,13 @@
         <v>465</v>
       </c>
       <c r="E83" s="3" t="s">
+        <v>835</v>
+      </c>
+      <c r="F83" s="3" t="s">
+        <v>836</v>
+      </c>
+      <c r="G83" s="9" t="s">
         <v>837</v>
-      </c>
-      <c r="F83" s="3" t="s">
-        <v>838</v>
-      </c>
-      <c r="G83" s="9" t="s">
-        <v>839</v>
       </c>
       <c r="H83" s="9" t="s">
         <v>252</v>
@@ -7866,13 +7845,13 @@
         <v>452</v>
       </c>
       <c r="E84" s="3" t="s">
+        <v>838</v>
+      </c>
+      <c r="F84" s="3" t="s">
+        <v>839</v>
+      </c>
+      <c r="G84" s="9" t="s">
         <v>840</v>
-      </c>
-      <c r="F84" s="3" t="s">
-        <v>841</v>
-      </c>
-      <c r="G84" s="9" t="s">
-        <v>842</v>
       </c>
       <c r="H84" s="9" t="s">
         <v>252</v>
@@ -7898,13 +7877,13 @@
         <v>472</v>
       </c>
       <c r="E85" s="3" t="s">
+        <v>841</v>
+      </c>
+      <c r="F85" s="3" t="s">
+        <v>842</v>
+      </c>
+      <c r="G85" s="9" t="s">
         <v>843</v>
-      </c>
-      <c r="F85" s="3" t="s">
-        <v>844</v>
-      </c>
-      <c r="G85" s="9" t="s">
-        <v>845</v>
       </c>
       <c r="H85" s="9" t="s">
         <v>252</v>
@@ -7930,13 +7909,13 @@
         <v>476</v>
       </c>
       <c r="E86" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="F86" s="3" t="s">
+        <v>845</v>
+      </c>
+      <c r="G86" s="9" t="s">
         <v>846</v>
-      </c>
-      <c r="F86" s="3" t="s">
-        <v>847</v>
-      </c>
-      <c r="G86" s="9" t="s">
-        <v>848</v>
       </c>
       <c r="H86" s="9" t="s">
         <v>252</v>
@@ -7962,13 +7941,13 @@
         <v>381</v>
       </c>
       <c r="E87" s="3" t="s">
+        <v>847</v>
+      </c>
+      <c r="F87" s="3" t="s">
+        <v>848</v>
+      </c>
+      <c r="G87" s="9" t="s">
         <v>849</v>
-      </c>
-      <c r="F87" s="3" t="s">
-        <v>850</v>
-      </c>
-      <c r="G87" s="9" t="s">
-        <v>851</v>
       </c>
       <c r="H87" s="9" t="s">
         <v>252</v>
@@ -7994,13 +7973,13 @@
         <v>484</v>
       </c>
       <c r="E88" s="3" t="s">
+        <v>850</v>
+      </c>
+      <c r="F88" s="3" t="s">
+        <v>851</v>
+      </c>
+      <c r="G88" s="9" t="s">
         <v>852</v>
-      </c>
-      <c r="F88" s="3" t="s">
-        <v>853</v>
-      </c>
-      <c r="G88" s="9" t="s">
-        <v>854</v>
       </c>
       <c r="H88" s="9" t="s">
         <v>252</v>
@@ -8026,13 +8005,13 @@
         <v>381</v>
       </c>
       <c r="E89" s="3" t="s">
+        <v>853</v>
+      </c>
+      <c r="F89" s="3" t="s">
+        <v>854</v>
+      </c>
+      <c r="G89" s="9" t="s">
         <v>855</v>
-      </c>
-      <c r="F89" s="3" t="s">
-        <v>856</v>
-      </c>
-      <c r="G89" s="9" t="s">
-        <v>857</v>
       </c>
       <c r="H89" s="9" t="s">
         <v>252</v>
@@ -8058,22 +8037,22 @@
         <v>490</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="F90" s="3" t="s">
         <v>491</v>
       </c>
       <c r="G90" s="9" t="s">
-        <v>945</v>
+        <v>940</v>
       </c>
       <c r="H90" s="9" t="s">
         <v>252</v>
       </c>
       <c r="I90" s="9" t="s">
-        <v>924</v>
+        <v>919</v>
       </c>
       <c r="J90" s="9" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
     </row>
     <row r="91" spans="1:10" ht="101.5" x14ac:dyDescent="0.35">
@@ -8090,13 +8069,13 @@
         <v>493</v>
       </c>
       <c r="E91" s="3" t="s">
+        <v>857</v>
+      </c>
+      <c r="F91" s="3" t="s">
+        <v>858</v>
+      </c>
+      <c r="G91" s="9" t="s">
         <v>859</v>
-      </c>
-      <c r="F91" s="3" t="s">
-        <v>860</v>
-      </c>
-      <c r="G91" s="9" t="s">
-        <v>861</v>
       </c>
       <c r="H91" s="9" t="s">
         <v>252</v>
@@ -8122,13 +8101,13 @@
         <v>309</v>
       </c>
       <c r="E92" s="3" t="s">
+        <v>860</v>
+      </c>
+      <c r="F92" s="3" t="s">
+        <v>861</v>
+      </c>
+      <c r="G92" s="9" t="s">
         <v>862</v>
-      </c>
-      <c r="F92" s="3" t="s">
-        <v>863</v>
-      </c>
-      <c r="G92" s="9" t="s">
-        <v>864</v>
       </c>
       <c r="H92" s="9" t="s">
         <v>252</v>
@@ -8154,13 +8133,13 @@
         <v>498</v>
       </c>
       <c r="E93" s="3" t="s">
+        <v>863</v>
+      </c>
+      <c r="F93" s="3" t="s">
+        <v>864</v>
+      </c>
+      <c r="G93" s="9" t="s">
         <v>865</v>
-      </c>
-      <c r="F93" s="3" t="s">
-        <v>866</v>
-      </c>
-      <c r="G93" s="9" t="s">
-        <v>867</v>
       </c>
       <c r="H93" s="9" t="s">
         <v>252</v>
@@ -8186,13 +8165,13 @@
         <v>501</v>
       </c>
       <c r="E94" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="F94" s="3" t="s">
+        <v>867</v>
+      </c>
+      <c r="G94" s="9" t="s">
         <v>868</v>
-      </c>
-      <c r="F94" s="3" t="s">
-        <v>869</v>
-      </c>
-      <c r="G94" s="9" t="s">
-        <v>870</v>
       </c>
       <c r="H94" s="9" t="s">
         <v>252</v>
@@ -8218,13 +8197,13 @@
         <v>505</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="F95" s="3" t="s">
         <v>506</v>
       </c>
       <c r="G95" s="9" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="H95" s="9" t="s">
         <v>252</v>
@@ -8236,33 +8215,33 @@
         <v>253</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A96" s="4" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>470</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>873</v>
+        <v>869</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>874</v>
+        <v>506</v>
       </c>
       <c r="G96" s="9" t="s">
-        <v>875</v>
+        <v>870</v>
       </c>
       <c r="H96" s="9" t="s">
         <v>252</v>
       </c>
       <c r="I96" s="9" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="J96" s="9" t="s">
         <v>253</v>
@@ -8276,28 +8255,28 @@
         <v>474</v>
       </c>
       <c r="C97" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="E97" s="3" t="s">
+        <v>871</v>
+      </c>
+      <c r="F97" s="3" t="s">
         <v>510</v>
       </c>
-      <c r="D97" s="3" t="s">
-        <v>511</v>
-      </c>
-      <c r="E97" s="3" t="s">
-        <v>876</v>
-      </c>
-      <c r="F97" s="3" t="s">
-        <v>512</v>
-      </c>
       <c r="G97" s="9" t="s">
-        <v>877</v>
+        <v>872</v>
       </c>
       <c r="H97" s="9" t="s">
         <v>252</v>
       </c>
       <c r="I97" s="9" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="J97" s="9" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
     </row>
     <row r="98" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
@@ -8308,19 +8287,19 @@
         <v>478</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>381</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>878</v>
+        <v>873</v>
       </c>
       <c r="F98" s="3" t="s">
-        <v>879</v>
+        <v>874</v>
       </c>
       <c r="G98" s="9" t="s">
-        <v>880</v>
+        <v>875</v>
       </c>
       <c r="H98" s="9" t="s">
         <v>252</v>
@@ -8340,19 +8319,19 @@
         <v>482</v>
       </c>
       <c r="C99" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="E99" s="3" t="s">
+        <v>876</v>
+      </c>
+      <c r="F99" s="3" t="s">
         <v>516</v>
       </c>
-      <c r="D99" s="3" t="s">
-        <v>517</v>
-      </c>
-      <c r="E99" s="3" t="s">
-        <v>881</v>
-      </c>
-      <c r="F99" s="3" t="s">
-        <v>518</v>
-      </c>
       <c r="G99" s="9" t="s">
-        <v>882</v>
+        <v>877</v>
       </c>
       <c r="H99" s="9" t="s">
         <v>252</v>
@@ -8372,28 +8351,28 @@
         <v>486</v>
       </c>
       <c r="C100" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="E100" s="3" t="s">
+        <v>878</v>
+      </c>
+      <c r="F100" s="3" t="s">
         <v>519</v>
       </c>
-      <c r="D100" s="3" t="s">
-        <v>520</v>
-      </c>
-      <c r="E100" s="3" t="s">
-        <v>883</v>
-      </c>
-      <c r="F100" s="3" t="s">
-        <v>521</v>
-      </c>
       <c r="G100" s="9" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
       <c r="H100" s="9" t="s">
         <v>252</v>
       </c>
       <c r="I100" s="9" t="s">
-        <v>925</v>
+        <v>920</v>
       </c>
       <c r="J100" s="9" t="s">
-        <v>948</v>
+        <v>943</v>
       </c>
     </row>
   </sheetData>
@@ -8455,1054 +8434,1054 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="175" x14ac:dyDescent="0.35" customHeight="1">
+    <row r="2" spans="1:11" ht="175" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>301</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>951</v>
+        <v>946</v>
       </c>
       <c r="D2" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>947</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H2" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>952</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H2" s="9" t="s">
+      <c r="I2" s="9" t="s">
+        <v>524</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K2" s="10" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="160" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="9" t="s">
         <v>525</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>526</v>
-      </c>
-      <c r="J2" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K2" s="10" t="s">
-        <v>953</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="160" x14ac:dyDescent="0.35" customHeight="1">
-      <c r="A3" s="9" t="s">
-        <v>527</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>342</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="D3" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>949</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="H3" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E3" s="10" t="s">
-        <v>954</v>
-      </c>
-      <c r="F3" s="9" t="s">
+      <c r="I3" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="G3" s="9" t="s">
-        <v>524</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I3" s="9" t="s">
+      <c r="J3" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="205" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
         <v>526</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K3" s="10" t="s">
-        <v>955</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="205" x14ac:dyDescent="0.35" customHeight="1">
-      <c r="A4" s="9" t="s">
-        <v>528</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>414</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>956</v>
+        <v>951</v>
       </c>
       <c r="D4" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>952</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H4" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>957</v>
-      </c>
-      <c r="F4" s="9" t="s">
+      <c r="I4" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="G4" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>526</v>
-      </c>
       <c r="J4" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="160" x14ac:dyDescent="0.35" customHeight="1">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="160" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>447</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>958</v>
+        <v>953</v>
       </c>
       <c r="D5" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>954</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="H5" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E5" s="10" t="s">
-        <v>959</v>
-      </c>
-      <c r="F5" s="9" t="s">
+      <c r="I5" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="G5" s="9" t="s">
-        <v>539</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>526</v>
-      </c>
       <c r="J5" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>960</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="175" x14ac:dyDescent="0.35" customHeight="1">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="175" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>453</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>961</v>
+        <v>956</v>
       </c>
       <c r="D6" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>957</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="H6" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E6" s="10" t="s">
-        <v>962</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G6" s="9" t="s">
+      <c r="I6" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="H6" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>526</v>
-      </c>
       <c r="J6" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>963</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="175" x14ac:dyDescent="0.35" customHeight="1">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="175" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>456</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>964</v>
+        <v>959</v>
       </c>
       <c r="D7" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>960</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="H7" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>965</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G7" s="9" t="s">
+      <c r="I7" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="H7" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>526</v>
-      </c>
       <c r="J7" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>966</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="145" x14ac:dyDescent="0.35" customHeight="1">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="145" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>459</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="D8" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>962</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="H8" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E8" s="10" t="s">
-        <v>967</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>539</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>539</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>525</v>
-      </c>
       <c r="I8" s="9" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="160" x14ac:dyDescent="0.35" customHeight="1">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="160" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>462</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>969</v>
+        <v>964</v>
       </c>
       <c r="D9" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>965</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H9" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>970</v>
-      </c>
-      <c r="F9" s="9" t="s">
+      <c r="I9" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="G9" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>526</v>
-      </c>
       <c r="J9" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>971</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="175" x14ac:dyDescent="0.35" customHeight="1">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="175" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>466</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="D10" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>967</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H10" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E10" s="10" t="s">
-        <v>972</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H10" s="9" t="s">
-        <v>525</v>
-      </c>
       <c r="I10" s="9" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="175" x14ac:dyDescent="0.35" customHeight="1">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="175" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>469</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="D11" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>968</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="H11" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E11" s="10" t="s">
-        <v>973</v>
-      </c>
-      <c r="F11" s="9" t="s">
+      <c r="I11" s="9" t="s">
+        <v>524</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="190" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="9" t="s">
         <v>539</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>539</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>526</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K11" s="10" t="s">
-        <v>974</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="190" x14ac:dyDescent="0.35" customHeight="1">
-      <c r="A12" s="9" t="s">
-        <v>541</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>473</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="D12" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H12" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E12" s="10" t="s">
-        <v>975</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>525</v>
-      </c>
       <c r="I12" s="9" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="145" x14ac:dyDescent="0.35" customHeight="1">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="145" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>477</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>976</v>
+        <v>971</v>
       </c>
       <c r="D13" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>972</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="H13" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E13" s="10" t="s">
-        <v>977</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>539</v>
-      </c>
-      <c r="G13" s="9" t="s">
+      <c r="I13" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="H13" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I13" s="9" t="s">
-        <v>526</v>
-      </c>
       <c r="J13" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="190" x14ac:dyDescent="0.35" customHeight="1">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="190" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>480</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>978</v>
+        <v>973</v>
       </c>
       <c r="D14" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>974</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="H14" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E14" s="10" t="s">
-        <v>979</v>
-      </c>
-      <c r="F14" s="9" t="s">
+      <c r="I14" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="G14" s="9" t="s">
-        <v>524</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I14" s="9" t="s">
-        <v>526</v>
-      </c>
       <c r="J14" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="175" x14ac:dyDescent="0.35" customHeight="1">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="175" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>485</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>980</v>
+        <v>975</v>
       </c>
       <c r="D15" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>976</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="H15" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E15" s="10" t="s">
-        <v>981</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G15" s="9" t="s">
-        <v>539</v>
-      </c>
-      <c r="H15" s="9" t="s">
-        <v>525</v>
-      </c>
       <c r="I15" s="9" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="175" x14ac:dyDescent="0.35" customHeight="1">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="175" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="B16" s="9" t="s">
         <v>488</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="D16" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>977</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H16" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E16" s="10" t="s">
-        <v>982</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G16" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H16" s="9" t="s">
-        <v>525</v>
-      </c>
       <c r="I16" s="9" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="160" x14ac:dyDescent="0.35" customHeight="1">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="160" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>494</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="D17" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>978</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H17" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E17" s="10" t="s">
-        <v>983</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>525</v>
-      </c>
       <c r="I17" s="9" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="175" x14ac:dyDescent="0.35" customHeight="1">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="175" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="B18" s="9" t="s">
         <v>496</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>984</v>
+        <v>979</v>
       </c>
       <c r="D18" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>980</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H18" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E18" s="10" t="s">
-        <v>985</v>
-      </c>
-      <c r="F18" s="9" t="s">
+      <c r="I18" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="G18" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I18" s="9" t="s">
-        <v>526</v>
-      </c>
       <c r="J18" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="130" x14ac:dyDescent="0.35" customHeight="1">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="130" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="9" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>499</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>986</v>
+        <v>981</v>
       </c>
       <c r="D19" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>982</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H19" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E19" s="10" t="s">
-        <v>987</v>
-      </c>
-      <c r="F19" s="9" t="s">
+      <c r="I19" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="G19" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H19" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I19" s="9" t="s">
-        <v>526</v>
-      </c>
       <c r="J19" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>988</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="160" x14ac:dyDescent="0.35" customHeight="1">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="160" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="9" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="B20" s="9" t="s">
         <v>502</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>989</v>
+        <v>984</v>
       </c>
       <c r="D20" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>985</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>646</v>
+      </c>
+      <c r="H20" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E20" s="10" t="s">
-        <v>990</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>648</v>
-      </c>
-      <c r="H20" s="9" t="s">
-        <v>525</v>
-      </c>
       <c r="I20" s="9" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="175" x14ac:dyDescent="0.35" customHeight="1">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="175" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="9" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="B21" s="9" t="s">
         <v>507</v>
       </c>
       <c r="C21" s="9" t="s">
+        <v>565</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>986</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>523</v>
+      </c>
+      <c r="I21" s="9" t="s">
+        <v>524</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K21" s="10" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="130" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="9" t="s">
+        <v>562</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>511</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>568</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>987</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>523</v>
+      </c>
+      <c r="I22" s="9" t="s">
+        <v>524</v>
+      </c>
+      <c r="J22" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K22" s="10" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="175" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="9" t="s">
+        <v>564</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>908</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>910</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>988</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>523</v>
+      </c>
+      <c r="I23" s="9" t="s">
+        <v>911</v>
+      </c>
+      <c r="J23" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K23" s="10" t="s">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="160" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="9" t="s">
         <v>567</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="B24" s="9" t="s">
+        <v>914</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>989</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>990</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H24" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="I24" s="9" t="s">
+        <v>524</v>
+      </c>
+      <c r="J24" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K24" s="10" t="s">
         <v>991</v>
       </c>
-      <c r="F21" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G21" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H21" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I21" s="9" t="s">
-        <v>526</v>
-      </c>
-      <c r="J21" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K21" s="10" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="130" x14ac:dyDescent="0.35" customHeight="1">
-      <c r="A22" s="9" t="s">
-        <v>564</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>513</v>
-      </c>
-      <c r="C22" s="9" t="s">
+    </row>
+    <row r="25" spans="1:11" ht="160" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="9" t="s">
         <v>570</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="B25" s="9" t="s">
+        <v>915</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>992</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>993</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H25" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E22" s="10" t="s">
-        <v>992</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>539</v>
-      </c>
-      <c r="G22" s="9" t="s">
-        <v>539</v>
-      </c>
-      <c r="H22" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I22" s="9" t="s">
-        <v>526</v>
-      </c>
-      <c r="J22" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K22" s="10" t="s">
+      <c r="I25" s="9" t="s">
+        <v>524</v>
+      </c>
+      <c r="J25" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K25" s="10" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="190" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="9" t="s">
         <v>571</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" ht="175" x14ac:dyDescent="0.35" customHeight="1">
-      <c r="A23" s="9" t="s">
-        <v>566</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>913</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>915</v>
-      </c>
-      <c r="D23" s="9" t="s">
+      <c r="B26" s="9" t="s">
+        <v>917</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>995</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>996</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H26" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E23" s="10" t="s">
-        <v>993</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>539</v>
-      </c>
-      <c r="G23" s="9" t="s">
-        <v>539</v>
-      </c>
-      <c r="H23" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I23" s="9" t="s">
-        <v>916</v>
-      </c>
-      <c r="J23" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K23" s="10" t="s">
-        <v>917</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="160" x14ac:dyDescent="0.35" customHeight="1">
-      <c r="A24" s="9" t="s">
-        <v>569</v>
-      </c>
-      <c r="B24" s="9" t="s">
+      <c r="I26" s="9" t="s">
+        <v>524</v>
+      </c>
+      <c r="J26" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K26" s="10" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="145" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="9" t="s">
+        <v>572</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>918</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>998</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>999</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>523</v>
+      </c>
+      <c r="I27" s="9" t="s">
+        <v>1000</v>
+      </c>
+      <c r="J27" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K27" s="10" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="160" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="9" t="s">
+        <v>573</v>
+      </c>
+      <c r="B28" s="9" t="s">
         <v>919</v>
       </c>
-      <c r="C24" s="9" t="s">
-        <v>994</v>
-      </c>
-      <c r="D24" s="9" t="s">
+      <c r="C28" s="9" t="s">
+        <v>1002</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>1003</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H28" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E24" s="10" t="s">
-        <v>995</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G24" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H24" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I24" s="9" t="s">
-        <v>526</v>
-      </c>
-      <c r="J24" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K24" s="10" t="s">
-        <v>996</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="160" x14ac:dyDescent="0.35" customHeight="1">
-      <c r="A25" s="9" t="s">
-        <v>572</v>
-      </c>
-      <c r="B25" s="9" t="s">
+      <c r="I28" s="9" t="s">
+        <v>1000</v>
+      </c>
+      <c r="J28" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K28" s="10" t="s">
+        <v>941</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="160" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="9" t="s">
+        <v>574</v>
+      </c>
+      <c r="B29" s="9" t="s">
         <v>920</v>
       </c>
-      <c r="C25" s="9" t="s">
-        <v>997</v>
-      </c>
-      <c r="D25" s="9" t="s">
+      <c r="C29" s="9" t="s">
+        <v>1004</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>1005</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H29" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E25" s="10" t="s">
-        <v>998</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G25" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H25" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I25" s="9" t="s">
-        <v>526</v>
-      </c>
-      <c r="J25" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K25" s="10" t="s">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="190" x14ac:dyDescent="0.35" customHeight="1">
-      <c r="A26" s="9" t="s">
-        <v>573</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>922</v>
-      </c>
-      <c r="C26" s="9" t="s">
+      <c r="I29" s="9" t="s">
         <v>1000</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="J29" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K29" s="10" t="s">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="175" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="9" t="s">
+        <v>575</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>928</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>1007</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>1008</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H30" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E26" s="10" t="s">
-        <v>1001</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G26" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H26" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I26" s="9" t="s">
-        <v>526</v>
-      </c>
-      <c r="J26" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K26" s="10" t="s">
-        <v>1002</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="145" x14ac:dyDescent="0.35" customHeight="1">
-      <c r="A27" s="9" t="s">
-        <v>574</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>923</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>1003</v>
-      </c>
-      <c r="D27" s="9" t="s">
+      <c r="I30" s="9" t="s">
+        <v>1000</v>
+      </c>
+      <c r="J30" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K30" s="10" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="175" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="9" t="s">
+        <v>576</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>931</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>1010</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>1011</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E27" s="10" t="s">
-        <v>1004</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G27" s="9" t="s">
-        <v>524</v>
-      </c>
-      <c r="H27" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I27" s="9" t="s">
-        <v>1005</v>
-      </c>
-      <c r="J27" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K27" s="10" t="s">
-        <v>1006</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="160" x14ac:dyDescent="0.35" customHeight="1">
-      <c r="A28" s="9" t="s">
-        <v>575</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>924</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>1007</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>523</v>
-      </c>
-      <c r="E28" s="10" t="s">
-        <v>1008</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G28" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H28" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I28" s="9" t="s">
-        <v>1005</v>
-      </c>
-      <c r="J28" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K28" s="10" t="s">
-        <v>946</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="160" x14ac:dyDescent="0.35" customHeight="1">
-      <c r="A29" s="9" t="s">
-        <v>576</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>925</v>
-      </c>
-      <c r="C29" s="9" t="s">
+      <c r="I31" s="9" t="s">
+        <v>1000</v>
+      </c>
+      <c r="J31" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="K31" s="10" t="s">
         <v>1009</v>
-      </c>
-      <c r="D29" s="9" t="s">
-        <v>523</v>
-      </c>
-      <c r="E29" s="10" t="s">
-        <v>1010</v>
-      </c>
-      <c r="F29" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G29" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H29" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I29" s="9" t="s">
-        <v>1005</v>
-      </c>
-      <c r="J29" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K29" s="10" t="s">
-        <v>1011</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="175" x14ac:dyDescent="0.35" customHeight="1">
-      <c r="A30" s="9" t="s">
-        <v>577</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>933</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>1012</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>523</v>
-      </c>
-      <c r="E30" s="10" t="s">
-        <v>1013</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="G30" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H30" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I30" s="9" t="s">
-        <v>1005</v>
-      </c>
-      <c r="J30" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K30" s="10" t="s">
-        <v>1014</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="175" x14ac:dyDescent="0.35" customHeight="1">
-      <c r="A31" s="9" t="s">
-        <v>578</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>936</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>1015</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>523</v>
-      </c>
-      <c r="E31" s="10" t="s">
-        <v>1016</v>
-      </c>
-      <c r="F31" s="9" t="s">
-        <v>524</v>
-      </c>
-      <c r="G31" s="9" t="s">
-        <v>529</v>
-      </c>
-      <c r="H31" s="9" t="s">
-        <v>525</v>
-      </c>
-      <c r="I31" s="9" t="s">
-        <v>1005</v>
-      </c>
-      <c r="J31" s="9" t="s">
-        <v>1017</v>
-      </c>
-      <c r="K31" s="10" t="s">
-        <v>1014</v>
       </c>
     </row>
   </sheetData>
@@ -9545,7 +9524,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>14</v>
@@ -9565,7 +9544,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>14</v>
@@ -9585,7 +9564,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>14</v>
@@ -9605,7 +9584,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>14</v>
@@ -9625,7 +9604,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>14</v>
@@ -9645,7 +9624,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>17</v>
@@ -9665,7 +9644,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>17</v>
@@ -9685,7 +9664,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>17</v>
@@ -9705,7 +9684,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>17</v>
@@ -9725,7 +9704,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>17</v>
@@ -9745,7 +9724,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>17</v>
@@ -9765,7 +9744,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>20</v>
@@ -9785,7 +9764,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>20</v>
@@ -9805,7 +9784,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>20</v>
@@ -9825,7 +9804,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>20</v>
@@ -9845,7 +9824,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>20</v>
@@ -9865,7 +9844,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>23</v>
@@ -9885,7 +9864,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>23</v>
@@ -9905,7 +9884,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>23</v>
@@ -9925,7 +9904,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>23</v>
@@ -9945,7 +9924,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>23</v>
@@ -9965,7 +9944,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>23</v>
@@ -9985,7 +9964,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>23</v>
@@ -10005,7 +9984,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>26</v>
@@ -10025,7 +10004,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="B26" s="7" t="s">
         <v>26</v>
@@ -10045,7 +10024,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="7" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>26</v>
@@ -10065,7 +10044,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="7" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>26</v>
@@ -10085,7 +10064,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="7" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>26</v>
@@ -10105,7 +10084,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="7" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="B30" s="7" t="s">
         <v>26</v>
@@ -10125,7 +10104,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="7" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B31" s="7" t="s">
         <v>26</v>
@@ -10145,7 +10124,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="7" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="B32" s="7" t="s">
         <v>29</v>
@@ -10165,7 +10144,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="7" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>29</v>
@@ -10185,7 +10164,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="7" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="B34" s="7" t="s">
         <v>29</v>
@@ -10205,7 +10184,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B35" s="7" t="s">
         <v>29</v>
@@ -10225,7 +10204,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B36" s="7" t="s">
         <v>29</v>
@@ -10245,7 +10224,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="7" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B37" s="7" t="s">
         <v>29</v>
@@ -10265,7 +10244,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="7" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="B38" s="7" t="s">
         <v>32</v>
@@ -10285,7 +10264,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="7" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B39" s="7" t="s">
         <v>32</v>
@@ -10305,7 +10284,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="7" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="B40" s="7" t="s">
         <v>32</v>
@@ -10325,7 +10304,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="7" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B41" s="7" t="s">
         <v>32</v>
@@ -10345,7 +10324,7 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="7" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="B42" s="7" t="s">
         <v>32</v>
@@ -10365,7 +10344,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="7" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="B43" s="7" t="s">
         <v>141</v>
@@ -10380,12 +10359,12 @@
         <v>321</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>920</v>
+        <v>915</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="7" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="B44" s="7" t="s">
         <v>141</v>
@@ -10405,7 +10384,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="7" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="B45" s="7" t="s">
         <v>141</v>
@@ -10425,7 +10404,7 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="7" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B46" s="7" t="s">
         <v>35</v>
@@ -10445,7 +10424,7 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="7" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="B47" s="7" t="s">
         <v>35</v>
@@ -10465,7 +10444,7 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="7" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="B48" s="7" t="s">
         <v>35</v>
@@ -10485,7 +10464,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="7" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="B49" s="7" t="s">
         <v>35</v>
@@ -10505,7 +10484,7 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="7" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B50" s="7" t="s">
         <v>35</v>
@@ -10525,7 +10504,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="7" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="B51" s="7" t="s">
         <v>35</v>
@@ -10545,7 +10524,7 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="7" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="B52" s="7" t="s">
         <v>35</v>
@@ -10565,7 +10544,7 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="7" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="B53" s="7" t="s">
         <v>38</v>
@@ -10585,7 +10564,7 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="7" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="B54" s="7" t="s">
         <v>38</v>
@@ -10600,12 +10579,12 @@
         <v>350</v>
       </c>
       <c r="F54" s="7" t="s">
-        <v>913</v>
+        <v>908</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="7" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="B55" s="7" t="s">
         <v>38</v>
@@ -10625,7 +10604,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="7" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B56" s="7" t="s">
         <v>38</v>
@@ -10645,7 +10624,7 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="7" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="B57" s="7" t="s">
         <v>38</v>
@@ -10665,7 +10644,7 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="7" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="B58" s="7" t="s">
         <v>41</v>
@@ -10685,7 +10664,7 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="7" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="B59" s="7" t="s">
         <v>41</v>
@@ -10705,7 +10684,7 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="7" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="B60" s="7" t="s">
         <v>41</v>
@@ -10720,12 +10699,12 @@
         <v>367</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>919</v>
+        <v>914</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="7" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="B61" s="7" t="s">
         <v>44</v>
@@ -10745,7 +10724,7 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="7" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="B62" s="7" t="s">
         <v>44</v>
@@ -10765,7 +10744,7 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="7" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="B63" s="7" t="s">
         <v>44</v>
@@ -10780,12 +10759,12 @@
         <v>376</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>933</v>
+        <v>928</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="7" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="B64" s="7" t="s">
         <v>44</v>
@@ -10800,12 +10779,12 @@
         <v>379</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>936</v>
+        <v>931</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="7" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="B65" s="7" t="s">
         <v>177</v>
@@ -10825,7 +10804,7 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="7" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="B66" s="7" t="s">
         <v>177</v>
@@ -10840,12 +10819,12 @@
         <v>385</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>922</v>
+        <v>917</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="7" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="B67" s="7" t="s">
         <v>177</v>
@@ -10865,7 +10844,7 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="7" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="B68" s="7" t="s">
         <v>46</v>
@@ -10885,7 +10864,7 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="7" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="B69" s="7" t="s">
         <v>46</v>
@@ -10905,13 +10884,13 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="7" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="B70" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>949</v>
+        <v>944</v>
       </c>
       <c r="D70" s="7" t="s">
         <v>182</v>
@@ -10920,12 +10899,12 @@
         <v>398</v>
       </c>
       <c r="F70" s="7" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="7" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="B71" s="7" t="s">
         <v>46</v>
@@ -10945,7 +10924,7 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="7" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="B72" s="7" t="s">
         <v>46</v>
@@ -10965,7 +10944,7 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="7" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="B73" s="7" t="s">
         <v>46</v>
@@ -10985,7 +10964,7 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="7" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="B74" s="7" t="s">
         <v>46</v>
@@ -11005,7 +10984,7 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="7" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="B75" s="7" t="s">
         <v>46</v>
@@ -11025,7 +11004,7 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="7" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="B76" s="7" t="s">
         <v>26</v>
@@ -11045,7 +11024,7 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="7" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="B77" s="7" t="s">
         <v>26</v>
@@ -11065,7 +11044,7 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" s="7" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B78" s="7" t="s">
         <v>46</v>
@@ -11085,7 +11064,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" s="7" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="B79" s="7" t="s">
         <v>46</v>
@@ -11105,7 +11084,7 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="7" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="B80" s="7" t="s">
         <v>46</v>
@@ -11125,7 +11104,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" s="7" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B81" s="7" t="s">
         <v>46</v>
@@ -11145,7 +11124,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" s="7" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="B82" s="7" t="s">
         <v>35</v>
@@ -11165,7 +11144,7 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" s="7" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="B83" s="7" t="s">
         <v>38</v>
@@ -11185,7 +11164,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" s="7" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="B84" s="7" t="s">
         <v>38</v>
@@ -11205,7 +11184,7 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" s="7" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="B85" s="7" t="s">
         <v>38</v>
@@ -11225,7 +11204,7 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" s="7" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="B86" s="7" t="s">
         <v>38</v>
@@ -11245,7 +11224,7 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" s="7" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="B87" s="7" t="s">
         <v>38</v>
@@ -11265,7 +11244,7 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" s="7" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="B88" s="7" t="s">
         <v>38</v>
@@ -11285,7 +11264,7 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" s="7" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="B89" s="7" t="s">
         <v>38</v>
@@ -11305,7 +11284,7 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" s="7" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="B90" s="7" t="s">
         <v>38</v>
@@ -11320,12 +11299,12 @@
         <v>450</v>
       </c>
       <c r="F90" s="7" t="s">
-        <v>924</v>
+        <v>919</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" s="7" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="B91" s="7" t="s">
         <v>17</v>
@@ -11345,7 +11324,7 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" s="7" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="B92" s="7" t="s">
         <v>29</v>
@@ -11365,7 +11344,7 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" s="7" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="B93" s="7" t="s">
         <v>29</v>
@@ -11385,7 +11364,7 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" s="7" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="B94" s="7" t="s">
         <v>44</v>
@@ -11405,7 +11384,7 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" s="7" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="B95" s="7" t="s">
         <v>26</v>
@@ -11425,7 +11404,7 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" s="7" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B96" s="7" t="s">
         <v>26</v>
@@ -11445,7 +11424,7 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" s="7" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="B97" s="7" t="s">
         <v>32</v>
@@ -11460,12 +11439,12 @@
         <v>474</v>
       </c>
       <c r="F97" s="7" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" s="7" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="B98" s="7" t="s">
         <v>177</v>
@@ -11485,7 +11464,7 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" s="7" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="B99" s="7" t="s">
         <v>177</v>
@@ -11505,7 +11484,7 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" s="7" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="B100" s="7" t="s">
         <v>177</v>
@@ -11520,7 +11499,7 @@
         <v>486</v>
       </c>
       <c r="F100" s="7" t="s">
-        <v>925</v>
+        <v>920</v>
       </c>
     </row>
   </sheetData>

</xml_diff>